<commit_message>
Fix Forge 60 LED board BOM part mapping
</commit_message>
<xml_diff>
--- a/forge60-hardware-release/led-board-5050/led-board-5050-bom.xlsx
+++ b/forge60-hardware-release/led-board-5050/led-board-5050-bom.xlsx
@@ -1,106 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet sheetId="1" name="BOM_5050灯板_PCB1_2_2026-06-20" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM_5050灯板_PCB1_2_2026-06-20" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
-  <si>
-    <t>No.</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>Designator</t>
-  </si>
-  <si>
-    <t>Footprint</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Manufacturer Part</t>
-  </si>
-  <si>
-    <t>Manufacturer</t>
-  </si>
-  <si>
-    <t>Supplier Part</t>
-  </si>
-  <si>
-    <t>Supplier</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>SAW9L60A</t>
-  </si>
-  <si>
-    <t>LED1,LED2,LED3,LED4,LED5,LED6,LED7,LED8,LED9,LED10,LED11,LED12,LED13,LED14,LED15,LED16,LED17,LED18,LED19,LED20,LED21,LED22,LED23,LED24,LED25,LED26,LED27,LED28,LED29,LED30,LED31,LED32</t>
-  </si>
-  <si>
-    <t>emc5050-1</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>KENTO</t>
-  </si>
-  <si>
-    <t>C34499</t>
-  </si>
-  <si>
-    <t>LCSC</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>SDNT1608X103F3435FTF</t>
-  </si>
-  <si>
-    <t>R1</t>
-  </si>
-  <si>
-    <t>R0603</t>
-  </si>
-  <si>
-    <t>Sunlord(顺络)</t>
-  </si>
-  <si>
-    <t>C525660</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <family val="2"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -119,21 +43,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -458,117 +441,161 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="10" width="20" customWidth="1"/>
+    <col width="20" customWidth="1" min="1" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Designator</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Footprint</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Manufacturer Part</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Manufacturer</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Supplier Part</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>32</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>STW0L8PA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LED1,LED2,LED3,LED4,LED5,LED6,LED7,LED8,LED9,LED10,LED11,LED12,LED13,LED14,LED15,LED16,LED17,LED18,LED19,LED20,LED21,LED22,LED23,LED24,LED25,LED26,LED27,LED28,LED29,LED30,LED31,LED32</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>emc5050-1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>6V 5050 white LED, 5700K, CRI 70</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>STW0L8PA</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Seoul Semiconductor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SDNT1608X103F3435FTF</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>R0603</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SDNT1608X103F3435FTF</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Sunlord(顺络)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>C525660</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LCSC</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
-        <v>32</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" t="s">
-        <v>23</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
     </row>
   </sheetData>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>